<commit_message>
fix: corrected data entry errors in 2024 survey datasheets
These were mostly just putting blank values in some cells that were assumed to take the value of the previous cell
</commit_message>
<xml_diff>
--- a/data_raw/data_raw_2024_sheets/LTER1_BR_P01_P10_2024.xlsx
+++ b/data_raw/data_raw_2024_sheets/LTER1_BR_P01_P10_2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/HLenihan/Documents/Work/Coral reefs/Demography study/Coral data/Demographic transect data/Data files/2024/Data 2024/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryananderson/Reference/Bren/Coral Demography/data_raw/data_raw_2024_sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9CC9F43-0C8D-4F48-AD72-BF8C330838E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6833CED8-421B-9941-8AF0-F8C4E7232E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="5880" windowWidth="37060" windowHeight="23500" xr2:uid="{8F4FB033-83A6-C940-818C-F60BB21E3E11}"/>
+    <workbookView xWindow="0" yWindow="560" windowWidth="29920" windowHeight="18780" xr2:uid="{8F4FB033-83A6-C940-818C-F60BB21E3E11}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="31">
   <si>
     <t>LTER1</t>
   </si>
@@ -206,7 +206,79 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="23">
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFA500"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFA500"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFA500"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2098,6 +2170,15 @@
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>0</v>
+      </c>
+      <c r="B41" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>12</v>
+      </c>
       <c r="D41" t="s">
         <v>3</v>
       </c>
@@ -2124,6 +2205,15 @@
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>0</v>
+      </c>
+      <c r="B42" t="s">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
+        <v>12</v>
+      </c>
       <c r="D42" t="s">
         <v>3</v>
       </c>
@@ -2153,6 +2243,15 @@
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>0</v>
+      </c>
+      <c r="B43" t="s">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
+        <v>12</v>
+      </c>
       <c r="D43" t="s">
         <v>3</v>
       </c>
@@ -2181,64 +2280,88 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="A2:H2">
-    <cfRule type="beginsWith" dxfId="16" priority="8" operator="beginsWith" text="FI">
+    <cfRule type="beginsWith" dxfId="22" priority="14" operator="beginsWith" text="FI">
       <formula>LEFT(A2,LEN("FI"))="FI"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="9" operator="containsText" text="Missing data">
+    <cfRule type="containsText" dxfId="21" priority="15" operator="containsText" text="Missing data">
       <formula>NOT(ISERROR(SEARCH("Missing data",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:M2">
-    <cfRule type="beginsWith" dxfId="14" priority="1" operator="beginsWith" text="UK">
+    <cfRule type="beginsWith" dxfId="20" priority="7" operator="beginsWith" text="UK">
       <formula>LEFT(A2,LEN("UK"))="UK"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="13" priority="7" operator="beginsWith" text="FU">
+    <cfRule type="beginsWith" dxfId="19" priority="13" operator="beginsWith" text="FU">
       <formula>LEFT(A2,LEN("FU"))="FU"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H23 H40">
-    <cfRule type="containsText" dxfId="12" priority="12" operator="containsText" text=",">
+    <cfRule type="containsText" dxfId="18" priority="18" operator="containsText" text=",">
       <formula>NOT(ISERROR(SEARCH(",", H3)))</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="11" priority="13" operator="beginsWith" text="Fusion">
+    <cfRule type="beginsWith" dxfId="17" priority="19" operator="beginsWith" text="Fusion">
       <formula>LEFT(H3,LEN("Fusion"))="Fusion"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="10" priority="14" operator="beginsWith" text="Fission">
+    <cfRule type="beginsWith" dxfId="16" priority="20" operator="beginsWith" text="Fission">
       <formula>LEFT(H3,LEN("Fission"))="Fission"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="15">
+    <cfRule type="expression" dxfId="15" priority="21">
       <formula>H3="Death"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="16">
+    <cfRule type="expression" dxfId="14" priority="22">
       <formula>H3="Growth"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="17">
+    <cfRule type="expression" dxfId="13" priority="23">
       <formula>H3="Recruitment"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3:K4 A3:H23 I6:K9 I11:K18 I20:K20 I22:K25 A24:G39 I27:K38 A40:K40 D41:G43 I41:K43">
-    <cfRule type="expression" dxfId="6" priority="10">
+    <cfRule type="expression" dxfId="12" priority="16">
       <formula>A3="UK"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="11">
+    <cfRule type="expression" dxfId="11" priority="17">
       <formula>A3="Na"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="beginsWith" dxfId="4" priority="2" operator="beginsWith" text="FI">
+    <cfRule type="beginsWith" dxfId="10" priority="8" operator="beginsWith" text="FI">
       <formula>LEFT(I2,LEN("FI"))="FI"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="Missing data">
+    <cfRule type="containsText" dxfId="9" priority="9" operator="containsText" text="Missing data">
       <formula>NOT(ISERROR(SEARCH("Missing data",I2)))</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="2" priority="4" operator="beginsWith" text="R">
+    <cfRule type="beginsWith" dxfId="8" priority="10" operator="beginsWith" text="R">
       <formula>LEFT(I2,LEN("R"))="R"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="NA">
+    <cfRule type="containsText" dxfId="7" priority="11" operator="containsText" text="NA">
       <formula>NOT(ISERROR(SEARCH("NA",I2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="D">
+    <cfRule type="containsText" dxfId="6" priority="12" operator="containsText" text="D">
       <formula>NOT(ISERROR(SEARCH("D",I2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A41:C41">
+    <cfRule type="expression" dxfId="5" priority="5">
+      <formula>A41="UK"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="6">
+      <formula>A41="Na"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A42:C42">
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>A42="UK"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="4">
+      <formula>A42="Na"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A43:C43">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>A43="UK"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>A43="Na"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions gridLines="1"/>

</xml_diff>